<commit_message>
Manage Email/Text to Pay-final
</commit_message>
<xml_diff>
--- a/KatalonData/EmailTextToPay/Manage_EmailText_1.xlsx
+++ b/KatalonData/EmailTextToPay/Manage_EmailText_1.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="69">
   <si>
     <t>Result</t>
   </si>
@@ -168,6 +168,81 @@
   </si>
   <si>
     <t>Thu Apr 09 21:27:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 13 17:10:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 13 17:17:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 13 17:19:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 18:00:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 18:06:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 18:17:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 18:21:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 18:59:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 19:05:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 19:09:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 19:42:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 19:59:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 20:16:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 21:08:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 21:11:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 21:23:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 21:27:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Apr 14 21:48:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 15 18:56:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 15 19:19:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 15 19:29:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 15 19:35:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 20 19:28:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 20 19:36:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 20 19:42:24 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -774,7 +849,7 @@
         <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
rearanged code for 'Manage Email Text To Pay' module
</commit_message>
<xml_diff>
--- a/KatalonData/EmailTextToPay/Manage_EmailText_1.xlsx
+++ b/KatalonData/EmailTextToPay/Manage_EmailText_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t470258\Documents\VPS-Katalon\KatalonData\EmailTextToPay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{B907D16B-99C1-456B-AA94-82A950A3052A}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr documentId="13_ncr:1_{A564B312-3550-40C5-87DD-24969108FEB6}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
     <workbookView windowHeight="11500" windowWidth="19420" xWindow="-110" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}" yWindow="-110"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="64">
   <si>
     <t>Result</t>
   </si>
@@ -152,145 +152,82 @@
     <t>Y</t>
   </si>
   <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Thu Apr 30 15:23:49 IST 2026</t>
+  </si>
+  <si>
+    <t>DueDate</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Tue Apr 07 21:52:12 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 08 16:55:05 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 08 17:09:19 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 09 21:27:28 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Apr 13 17:10:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Apr 13 17:17:06 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Apr 13 17:19:09 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 18:00:15 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 18:06:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 18:17:46 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 18:21:57 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 18:59:59 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 19:05:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 19:09:16 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 19:42:16 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 19:59:43 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 20:16:13 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 21:08:43 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 21:11:38 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 21:23:05 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 21:27:53 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Apr 14 21:48:14 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 15 18:56:56 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 15 19:19:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 15 19:29:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Apr 15 19:35:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Apr 20 19:28:12 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Apr 20 19:36:27 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Apr 20 19:42:24 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 14:57:01 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 14:58:08 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 14:59:14 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:12:35 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:13:36 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:14:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:15:33 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:16:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:17:15 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:18:05 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:18:57 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:19:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:20:56 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:21:57 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:22:54 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Apr 30 15:23:49 IST 2026</t>
+    <t>Mon May 11 18:52:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 18:59:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:04:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:09:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:19:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:22:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:25:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:27:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:30:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:32:28 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:35:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:37:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:40:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:44:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:47:10 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:49:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon May 11 19:52:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue May 12 15:21:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue May 12 18:06:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Tue May 12 18:41:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed May 13 12:56:59 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -410,7 +347,7 @@
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
     <xf applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="4" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
     <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
@@ -450,6 +387,9 @@
     </xf>
     <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf applyAlignment="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="3" numFmtId="49" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -786,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F033DD18-DD0F-43E3-A2D0-6223D1731E2C}">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="6.26953125" collapsed="true"/>
@@ -800,16 +740,17 @@
     <col min="10" max="10" customWidth="true" style="6" width="17.7265625" collapsed="true"/>
     <col min="11" max="11" customWidth="true" style="6" width="11.90625" collapsed="true"/>
     <col min="12" max="12" customWidth="true" style="6" width="15.0" collapsed="true"/>
-    <col min="13" max="14" customWidth="true" style="6" width="14.453125" collapsed="true"/>
-    <col min="15" max="15" customWidth="true" style="6" width="7.81640625" collapsed="true"/>
-    <col min="16" max="16" customWidth="true" style="6" width="9.1796875" collapsed="true"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" style="6" width="13.90625" collapsed="true"/>
-    <col min="18" max="18" customWidth="true" style="6" width="8.54296875" collapsed="true"/>
-    <col min="19" max="27" style="6" width="8.7265625" collapsed="true"/>
-    <col min="28" max="16384" style="1" width="8.7265625" collapsed="true"/>
+    <col min="13" max="13" customWidth="true" style="6" width="11.7265625" collapsed="true"/>
+    <col min="14" max="15" customWidth="true" style="6" width="14.453125" collapsed="true"/>
+    <col min="16" max="16" customWidth="true" style="6" width="7.81640625" collapsed="true"/>
+    <col min="17" max="17" customWidth="true" style="6" width="9.1796875" collapsed="true"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="6" width="13.90625" collapsed="true"/>
+    <col min="19" max="19" customWidth="true" style="6" width="8.54296875" collapsed="true"/>
+    <col min="20" max="28" style="6" width="8.7265625" collapsed="true"/>
+    <col min="29" max="16384" style="1" width="8.7265625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row customFormat="1" ht="25" r="1" s="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row customFormat="1" ht="25" r="1" s="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -847,57 +788,60 @@
         <v>20</v>
       </c>
       <c r="M1" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="R1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="V1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="W1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Y1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Z1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AA1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="AA1" s="9" t="s">
+      <c r="AB1" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row ht="25" r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row ht="25" r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>36</v>
@@ -914,28 +858,31 @@
       <c r="K2" s="6">
         <v>1234567890</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="P2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="6">
+      <c r="Q2" s="6">
         <v>123456</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="R2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="S2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="S2" s="6" t="s">
+      <c r="T2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="T2" s="6" t="s">
+      <c r="U2" s="6" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>